<commit_message>
fix: COM_Inventory 讀 role.json 初始裝備/背包時漏了 inv 這一層
role.json 的裝備/背包資料包在 inv 底下(inv.equips/inv.storage)，但
COM_Inventory.bind() 讀的是 bb.meta?.storage/bb.meta?.equips，少了中間的
.inv，永遠讀到 undefined，NPC 在 role.json 定義的初始裝備從未生效
(例如 rogue 的 sword_01)。npc.js 啟用元件時的判斷式 bb.meta.inv!==undefined
本身是對的，只有元件內部讀資料漏了這一層。

改成 bb.meta?.inv?.storage / bb.meta?.inv?.equips。

xls/role.xlsx 同步新增 rogue-2(配 bow_01)用來驗證近戰/遠程武器都能正確帶出來，
重新跑 node scripts/role.js 產生 role.json。
</commit_message>
<xml_diff>
--- a/xls/role.xlsx
+++ b/xls/role.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="15" windowWidth="19200" windowHeight="11760" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="15" windowWidth="19200" windowHeight="11760" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="player" state="visible" r:id="rId4"/>
-    <sheet sheetId="4" name="brooklyn" state="visible" r:id="rId5"/>
-    <sheet sheetId="5" name="rogues" state="visible" r:id="rId6"/>
-    <sheet sheetId="2" name="monsters" state="visible" r:id="rId7"/>
-    <sheet sheetId="6" name="animals" state="visible" r:id="rId8"/>
+    <sheet name="player" sheetId="1" r:id="rId1"/>
+    <sheet name="brooklyn" sheetId="4" r:id="rId2"/>
+    <sheet name="rogues" sheetId="5" r:id="rId3"/>
+    <sheet name="monsters" sheetId="2" r:id="rId4"/>
+    <sheet name="animals" sheetId="6" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="139">
   <si>
     <t>id</t>
   </si>
@@ -41,7 +41,7 @@
     <t>_view</t>
   </si>
   <si>
-    <t xml:space="preserve">"faceR":true,
+    <t>"faceR":true,
 "anchor":{"x":0,"y":16}, 
 "w":32, "h":64,
 "b":{"l":0,"r":0,"t":32,"b":0},
@@ -52,7 +52,7 @@
     <t>_shape</t>
   </si>
   <si>
-    <t xml:space="preserve">"body":{"sprite":"body-man","scale":0.25,"y":32},
+    <t>"body":{"sprite":"body-man","scale":0.25,"y":32},
 "hand":{"sprite":"hand-man","scale":0.25,"y":32},
 "head":{"sprite":"head-wick","scale":0.25,"y":3.5},
 "corpse":{"sprite":"rip","scale":0.5,"y":32}</t>
@@ -118,39 +118,39 @@
     <t>"job":"trader","gold":200,"style":"weak","trade":true</t>
   </si>
   <si>
-    <t xml:space="preserve">"job":"butcher","gold":200,
+    <t>"job":"butcher","gold":200,
 "abilities":["fireball","heal"],"meat":"raw_meat","trade":true</t>
   </si>
   <si>
     <t>"job":"merchant","gold":200,"trade":true</t>
   </si>
   <si>
-    <t xml:space="preserve">"body":{"sprite":"trump","scale":0.25,"y":32},
+    <t>"body":{"sprite":"trump","scale":0.25,"y":32},
 "corpse":{"sprite":"rip","scale":0.5,"y":32}</t>
   </si>
   <si>
-    <t xml:space="preserve">"body":{"sprite":"melanie","scale":0.25,"y":32},
+    <t>"body":{"sprite":"melanie","scale":0.25,"y":32},
 "corpse":{"sprite":"rip","scale":0.5,"y":32}</t>
   </si>
   <si>
-    <t xml:space="preserve">"body":{"sprite":"musk","scale":0.25,"y":32},
+    <t>"body":{"sprite":"musk","scale":0.25,"y":32},
 "hand":{"sprite":"hand-man","scale":0.25,"y":32},
 "corpse":{"sprite":"rip","scale":0.5,"y":32}</t>
   </si>
   <si>
-    <t xml:space="preserve">"body":{"sprite":"xi","scale":0.25,"y":32},
+    <t>"body":{"sprite":"xi","scale":0.25,"y":32},
 "corpse":{"sprite":"rip","scale":0.5,"y":32}</t>
   </si>
   <si>
-    <t xml:space="preserve">"body":{"sprite":"macron","scale":0.25,"y":32},
+    <t>"body":{"sprite":"macron","scale":0.25,"y":32},
 "corpse":{"sprite":"rip","scale":0.5,"y":32}</t>
   </si>
   <si>
-    <t xml:space="preserve">"storage":{"capacity":-1,
+    <t>"storage":{"capacity":-1,
 "items":["sword_01",{"id":"helmet_01","count":1}]}</t>
   </si>
   <si>
-    <t xml:space="preserve">"storage":{"capacity":-1,
+    <t>"storage":{"capacity":-1,
 "items":["sword_01","chest_01","gloves_01","chest_02",{"id":"helmet_01","count":1}]}</t>
   </si>
   <si>
@@ -388,31 +388,23 @@
     <t>"t":"20:30~07:40", "p":"bed", "map":"m_04x05/macron-home"</t>
   </si>
   <si>
-    <t>rogue</t>
-  </si>
-  <si>
     <t>"job":"rogue","gold":200,"type":"enemy"</t>
   </si>
   <si>
-    <t xml:space="preserve">"body":{"sprite":"rogue","scale":0.25,"y":32},
-"hand":{"sprite":"hand-man","scale":0.25,"y":32},
-"corpse":{"sprite":"rip","scale":0.5,"y":32}</t>
-  </si>
-  <si>
     <t>"equips":["sword_01"]</t>
   </si>
   <si>
     <t>attrs</t>
   </si>
   <si>
-    <t xml:space="preserve">"attack": 5,
+    <t>"attack": 5,
 "defense": 0</t>
   </si>
   <si>
     <t>states</t>
   </si>
   <si>
-    <t xml:space="preserve">"life": {"cur":50,"max":50},
+    <t>"life": {"cur":50,"max":50},
 "hunger": {"cur":0,"max":100},
 "thirst": {"cur":0,"max":100}</t>
   </si>
@@ -423,7 +415,7 @@
     <t>monsters:0</t>
   </si>
   <si>
-    <t xml:space="preserve">"faceR":false,
+    <t>"faceR":false,
 "anchor":{"x":-16,"y":16}, 
 "w":64, "h":64,
 "b":{"l":0,"r":0,"t":32,"b":0},
@@ -431,7 +423,7 @@
 "z":{"l":0,"r":0,"t":32,"b":0}</t>
   </si>
   <si>
-    <t xml:space="preserve">"body":{"sprite":"monsters:0","scale":2,"y":32},
+    <t>"body":{"sprite":"monsters:0","scale":2,"y":32},
 "corpse":{"sprite":"rip","scale":0.5,"y":32}</t>
   </si>
   <si>
@@ -453,35 +445,60 @@
     <t>"meat":"raw_meat","style":"skittish"</t>
   </si>
   <si>
-    <t xml:space="preserve">"body":{"sprite":"animals:42","scale":2,"y":32},
+    <t>"body":{"sprite":"animals:42","scale":2,"y":32},
 "corpse":{"sprite":"rip","scale":0.5,"y":32}</t>
   </si>
   <si>
-    <t xml:space="preserve">"body":{"sprite":"animals:82","scale":2,"y":32},
+    <t>"body":{"sprite":"animals:82","scale":2,"y":32},
 "corpse":{"sprite":"rip","scale":0.5,"y":32}</t>
+  </si>
+  <si>
+    <t>"body":{"sprite":"rogue","scale":0.25,"y":32},
+"hand":{"sprite":"hand-man","scale":0.25,"y":32},
+"corpse":{"sprite":"rip","scale":0.5,"y":32}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>rogue-1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>rogue-2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>"equips":["bow_01"]</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.00_ "/>
+    <numFmt numFmtId="176" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="新細明體"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="微軟正黑體 Light"/>
+      <family val="2"/>
       <charset val="136"/>
-      <color theme="1"/>
-      <family val="2"/>
-      <sz val="12"/>
-      <name val="微軟正黑體 Light"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="新細明體"/>
+      <family val="3"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -512,12 +529,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -816,16 +833,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.85546875" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="10.5703125" style="1" customWidth="1"/>
     <col min="2" max="2" width="52.85546875" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -833,7 +851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -841,7 +859,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -849,7 +867,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" ht="94.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="94.5" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -857,7 +875,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" ht="63" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="63" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -865,7 +883,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -873,7 +891,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -881,99 +899,23 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B8" s="3"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="200" verticalDpi="200"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="16.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="9.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="63" style="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="2" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="3" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="4" ht="94.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="5" ht="31.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="6" ht="31.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="7" ht="47.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="8" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="3"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G23"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.85546875" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="66" style="1" customWidth="1"/>
@@ -982,10 +924,11 @@
     <col min="5" max="5" width="75" style="1" customWidth="1"/>
     <col min="6" max="6" width="67.85546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="70.5703125" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.85546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1008,7 +951,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1031,7 +974,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="31.5" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1054,7 +997,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" ht="94.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="94.5" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1077,7 +1020,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" ht="47.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="47.25" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -1100,7 +1043,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" ht="31.5" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="31.5" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1120,7 +1063,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1143,7 +1086,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1166,7 +1109,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
@@ -1189,7 +1132,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
@@ -1212,7 +1155,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="A11" s="1" t="s">
         <v>14</v>
       </c>
@@ -1235,7 +1178,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="A12" s="1" t="s">
         <v>14</v>
       </c>
@@ -1258,7 +1201,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
@@ -1281,7 +1224,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="A14" s="1" t="s">
         <v>14</v>
       </c>
@@ -1301,7 +1244,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -1321,7 +1264,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -1338,7 +1281,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7">
       <c r="A17" s="1" t="s">
         <v>14</v>
       </c>
@@ -1355,7 +1298,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7">
       <c r="A18" s="1" t="s">
         <v>14</v>
       </c>
@@ -1372,7 +1315,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7">
       <c r="A19" s="1" t="s">
         <v>14</v>
       </c>
@@ -1389,7 +1332,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7">
       <c r="A20" s="1" t="s">
         <v>14</v>
       </c>
@@ -1406,7 +1349,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7">
       <c r="A21" s="1" t="s">
         <v>14</v>
       </c>
@@ -1423,7 +1366,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7">
       <c r="A22" s="1" t="s">
         <v>14</v>
       </c>
@@ -1440,7 +1383,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7">
       <c r="A23" s="1" t="s">
         <v>14</v>
       </c>
@@ -1458,182 +1401,288 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="16.5" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="56.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="54.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="94.5" customHeight="1">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="47.25" customHeight="1">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="31.5" customHeight="1">
+      <c r="A7" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="47.25" customHeight="1">
+      <c r="A8" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="3"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="16.5" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="63" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="94.5" customHeight="1">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="31.5" customHeight="1">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="31.5" customHeight="1">
+      <c r="A6" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="47.25" customHeight="1">
+      <c r="A7" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="15.75" customHeight="1">
+      <c r="A8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="3"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="200" verticalDpi="200"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="16.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="9.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="45.85546875" style="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="2" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="4" ht="94.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" ht="47.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="6" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="7" ht="31.5" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="8" ht="47.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="9" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="3"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="16.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="9.85546875" style="1" customWidth="1"/>
     <col min="2" max="3" width="63" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="2" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="3" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="4" ht="94.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="94.5" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="5" ht="31.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="31.5" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="6" ht="31.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="31.5" customHeight="1">
       <c r="A6" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="47.25" customHeight="1">
+      <c r="A7" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="7" ht="47.25" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="8" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="15.75" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1641,6 +1690,7 @@
       <c r="C8" s="3"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>